<commit_message>
Add Group 12: Amazon KDP project submission
</commit_message>
<xml_diff>
--- a/Group-List.xlsx
+++ b/Group-List.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -823,6 +823,38 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Group 12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Saurabh Yadav, Shashank Singh, Ankit Kumar, Ayush Khuntiya, Ashutosh Kumar Anand</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Amazon KDP</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Groups/Group-12/README.md</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Groups/Group-12/Presentation.pdf</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>